<commit_message>
Mise à jour valuebets 2025-07-08 03:21:39
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -498,10 +498,8 @@
           <t>11/07 21:30</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>55.00</t>
-        </is>
+      <c r="F2" t="n">
+        <v>55</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -516,7 +514,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -538,10 +536,8 @@
           <t>08/07 13:40</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>70.00</t>
-        </is>
+      <c r="F3" t="n">
+        <v>70</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -556,7 +552,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -578,10 +574,8 @@
           <t>12/07 14:00</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
+      <c r="F4" t="n">
+        <v>60</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -596,7 +590,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -618,10 +612,8 @@
           <t>12/07 21:00</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F5" t="n">
+        <v>45</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -636,7 +628,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -658,10 +650,8 @@
           <t>12/07 19:00</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F6" t="n">
+        <v>45</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -676,7 +666,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -698,10 +688,8 @@
           <t>13/07 14:30</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
+      <c r="F7" t="n">
+        <v>60</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -716,7 +704,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -738,10 +726,8 @@
           <t>12/07 15:30</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>55.00</t>
-        </is>
+      <c r="F8" t="n">
+        <v>55</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -756,7 +742,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -778,10 +764,8 @@
           <t>12/07 18:30</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F9" t="n">
+        <v>40</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -796,7 +780,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -818,10 +802,8 @@
           <t>09/07 19:00</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
+      <c r="F10" t="n">
+        <v>3.3</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -836,7 +818,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -858,10 +840,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2.18</t>
-        </is>
+      <c r="F11" t="n">
+        <v>2.18</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -876,7 +856,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -898,10 +878,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F12" t="n">
+        <v>40</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -916,7 +894,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -938,10 +916,8 @@
           <t>08/07 15:30</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F13" t="n">
+        <v>40</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -956,7 +932,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -978,10 +954,8 @@
           <t>08/07 12:00</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>1.60</t>
-        </is>
+      <c r="F14" t="n">
+        <v>1.6</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -996,7 +970,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1018,10 +992,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2.95</t>
-        </is>
+      <c r="F15" t="n">
+        <v>2.95</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1036,7 +1008,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1058,10 +1030,8 @@
           <t>08/07 18:00</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>1.24</t>
-        </is>
+      <c r="F16" t="n">
+        <v>1.24</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1076,7 +1046,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1098,10 +1068,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
+      <c r="F17" t="n">
+        <v>1.11</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1116,7 +1084,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1138,10 +1106,8 @@
           <t>09/07 03:00</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>2.05</t>
-        </is>
+      <c r="F18" t="n">
+        <v>2.05</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1156,7 +1122,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1178,10 +1144,8 @@
           <t>08/07 17:00</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F19" t="n">
+        <v>45</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1196,7 +1160,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1218,10 +1182,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>1.04</t>
-        </is>
+      <c r="F20" t="n">
+        <v>1.04</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1236,7 +1198,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1258,10 +1220,8 @@
           <t>09/07 17:30</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
+      <c r="F21" t="n">
+        <v>1.1</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1276,7 +1236,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1298,10 +1258,8 @@
           <t>09/07 17:30</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>1.04</t>
-        </is>
+      <c r="F22" t="n">
+        <v>1.04</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1316,7 +1274,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1338,10 +1296,8 @@
           <t>08/07 15:00</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
+      <c r="F23" t="n">
+        <v>1.11</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1356,7 +1312,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1378,10 +1334,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>1.16</t>
-        </is>
+      <c r="F24" t="n">
+        <v>1.16</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1396,7 +1350,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>45846.07739796837</v>
+        <v>45846.07739796296</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1418,10 +1372,8 @@
           <t>08/07 18:00</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
+      <c r="F25" t="n">
+        <v>1.15</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1431,6 +1383,246 @@
       <c r="H25" t="inlineStr">
         <is>
           <t>+0,56%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>45846.13996399079</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>KF Drita – FC Differdange 03Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Plus que 2.52e équipe</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>08/07 18:00</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>55.00</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2,33%</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>+28,4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>45846.13996399079</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Malmo FF – NorrkopingAllsvenskan stq pr cu 385076e7</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Plus que 3.52e équipe</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>12/07 15:30</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>55.00</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2,11%</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>+16,2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>45846.13996399079</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Cameron Norrie – Carlos AlcarazATP - Wimbledon</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Plus que 4.5 - break2e participant</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>08/07 13:40</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2.40</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>47,8%</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>+14,6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>45846.13996399079</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PMU(FR)Football</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>KF Egnatia Rrogozhine – BreidablikEurope. Ligue des Champions (Q)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>11-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>49,4%</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>+3,80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>45846.13996399079</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bwin(FR)Football</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Fotbal Club FCSB – Inter Club d'EscaldesEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2 / HNB</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>09/07 17:30</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>24,1%</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>+1,05%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>45846.13996399079</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Football</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>FC Noah – Buducnost PodgoricaEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>08/07 16:00</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1.19</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>84,9%</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>+1,04%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 05:23:39
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1388,7 +1388,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>45846.13996399079</v>
+        <v>45846.13996399305</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1410,10 +1410,8 @@
           <t>08/07 18:00</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>55.00</t>
-        </is>
+      <c r="F26" t="n">
+        <v>55</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1428,7 +1426,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>45846.13996399079</v>
+        <v>45846.13996399305</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1450,10 +1448,8 @@
           <t>12/07 15:30</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>55.00</t>
-        </is>
+      <c r="F27" t="n">
+        <v>55</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1468,7 +1464,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>45846.13996399079</v>
+        <v>45846.13996399305</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1490,10 +1486,8 @@
           <t>08/07 13:40</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>2.40</t>
-        </is>
+      <c r="F28" t="n">
+        <v>2.4</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1508,7 +1502,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>45846.13996399079</v>
+        <v>45846.13996399305</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1530,10 +1524,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
+      <c r="F29" t="n">
+        <v>2.1</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1548,7 +1540,7 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>45846.13996399079</v>
+        <v>45846.13996399305</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1570,10 +1562,8 @@
           <t>09/07 17:30</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
+      <c r="F30" t="n">
+        <v>4.2</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1588,7 +1578,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>45846.13996399079</v>
+        <v>45846.13996399305</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1610,10 +1600,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>1.19</t>
-        </is>
+      <c r="F31" t="n">
+        <v>1.19</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1623,6 +1611,126 @@
       <c r="H31" t="inlineStr">
         <is>
           <t>+1,04%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>45846.2246435659</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Cameron Norrie – Carlos AlcarazATP - Wimbledon</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Moins que 4.5 - break</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>08/07 13:40</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2.60</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>40,9%</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>+6,46%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>45846.2246435659</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>New England Revolution – Inter Miami CFÉtats-Unis - États-Unis MLS</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Moins que 8.5 - tir cadré</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>09/07 23:30</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2.65</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>39,9%</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>+5,78%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>45846.2246435659</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Football</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Egnatia Rrogozhine – Breidablik KopavogurEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>11-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>51,2%</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>+2,45%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 06:34:20
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1616,7 +1616,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>45846.2246435659</v>
+        <v>45846.22464356481</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1638,10 +1638,8 @@
           <t>08/07 13:40</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2.60</t>
-        </is>
+      <c r="F32" t="n">
+        <v>2.6</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1656,7 +1654,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>45846.2246435659</v>
+        <v>45846.22464356481</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1678,10 +1676,8 @@
           <t>09/07 23:30</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2.65</t>
-        </is>
+      <c r="F33" t="n">
+        <v>2.65</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1696,7 +1692,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>45846.2246435659</v>
+        <v>45846.22464356481</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1718,10 +1714,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
+      <c r="F34" t="n">
+        <v>2</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1731,6 +1725,166 @@
       <c r="H34" t="inlineStr">
         <is>
           <t>+2,45%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>45846.2737790988</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Cameron Norrie – Carlos AlcarazATP - Wimbledon</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Plus que 9.5 - aces2e participant</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>08/07 13:40</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>79,5%</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>+27,2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>45846.2737790988</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Football</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Fluminense – ChelseaInternational - CDM des Clubs</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Moins que 21.5 - tirs</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>37,3%</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>+19,2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>45846.2737790988</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Taylor Fritz – Karen KhachanovATP - Wimbledon</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1 - aces</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>08/07 12:00</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>91,9%</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>+1,13%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>45846.2737790988</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Football</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Levadia Tallinn – Rigas Futbola SkolaEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>08/07 16:30</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>75,9%</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>+0,23%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 07:22:52
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1730,7 +1730,7 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>45846.2737790988</v>
+        <v>45846.27377909722</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1752,10 +1752,8 @@
           <t>08/07 13:40</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>1.60</t>
-        </is>
+      <c r="F35" t="n">
+        <v>1.6</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1770,7 +1768,7 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>45846.2737790988</v>
+        <v>45846.27377909722</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1792,10 +1790,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
+      <c r="F36" t="n">
+        <v>3.2</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1810,7 +1806,7 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>45846.2737790988</v>
+        <v>45846.27377909722</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1832,10 +1828,8 @@
           <t>08/07 12:00</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
+      <c r="F37" t="n">
+        <v>1.1</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1850,7 +1844,7 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>45846.2737790988</v>
+        <v>45846.27377909722</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1872,10 +1866,8 @@
           <t>08/07 16:30</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>1.32</t>
-        </is>
+      <c r="F38" t="n">
+        <v>1.32</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1885,6 +1877,206 @@
       <c r="H38" t="inlineStr">
         <is>
           <t>+0,23%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>45846.3074425485</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Sportivo Ameliano – Cerro PortenoPrimera Division stq pr cu 385076e7</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Plus que 3.51re équipe</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>12/07 18:30</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2,82%</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>+12,6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>45846.3074425485</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ParionsSport(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>T.Fritz – K.KhachanovATP - Wimbledon H</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Moins que 21.5 - aces1er participant</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>08/07 12:00</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>50,0%</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>+7,50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>45846.3074425485</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Paris SG – Real MadridCoupe du Monde des Clubs</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Moins que 23.5 - tirs</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>09/07 19:00</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>34,4%</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>+3,29%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>45846.3074425485</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Levadia Tallinn – Rigas Futbola SkolaLigue des Champions</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2 / DNB</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>08/07 16:30</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>1.44</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>71,5%</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>+2,93%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>45846.3074425485</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Football</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Žalgiris – Hamrun SpartansEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>09/07 16:00</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>81,3%</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>+0,01%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 08:31:16
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1882,7 +1882,7 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>45846.3074425485</v>
+        <v>45846.3074425463</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1904,10 +1904,8 @@
           <t>12/07 18:30</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F39" t="n">
+        <v>40</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1922,7 +1920,7 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>45846.3074425485</v>
+        <v>45846.3074425463</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1944,10 +1942,8 @@
           <t>08/07 12:00</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>2.15</t>
-        </is>
+      <c r="F40" t="n">
+        <v>2.15</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1962,7 +1958,7 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>45846.3074425485</v>
+        <v>45846.3074425463</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1984,10 +1980,8 @@
           <t>09/07 19:00</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
+      <c r="F41" t="n">
+        <v>3</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2002,7 +1996,7 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>45846.3074425485</v>
+        <v>45846.3074425463</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2024,10 +2018,8 @@
           <t>08/07 16:30</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>1.44</t>
-        </is>
+      <c r="F42" t="n">
+        <v>1.44</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2042,7 +2034,7 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>45846.3074425485</v>
+        <v>45846.3074425463</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2064,10 +2056,8 @@
           <t>09/07 16:00</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>1.23</t>
-        </is>
+      <c r="F43" t="n">
+        <v>1.23</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2077,6 +2067,86 @@
       <c r="H43" t="inlineStr">
         <is>
           <t>+0,01%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>45846.35498854663</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>FC Iberia 1999 – Malmo FFLigue des Champions</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Plus que 3.51re équipe</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>08/07 16:00</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>1,59%</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>+59,0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>45846.35498854663</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Football</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Egnatia Rrogozhine – Breidablik KopavogurEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>80,7%</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>+0,11%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 09:26:42
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2072,7 +2072,7 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>45846.35498854663</v>
+        <v>45846.35498854167</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2094,10 +2094,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>100.00</t>
-        </is>
+      <c r="F44" t="n">
+        <v>100</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2112,7 +2110,7 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>45846.35498854663</v>
+        <v>45846.35498854167</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -2134,10 +2132,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>1.24</t>
-        </is>
+      <c r="F45" t="n">
+        <v>1.24</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2147,6 +2143,126 @@
       <c r="H45" t="inlineStr">
         <is>
           <t>+0,11%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45846.39348122294</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>PokerStars(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Arevalo/Pavic – Nys/Roger-VasselinWimbledon 2025 - Hommes</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>H 2 (+3.5)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>08/07 11:30</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>60,3%</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>+3,75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>45846.39348122294</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Volleyball</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Bulgarie (F) – Brésil (F)International - Ligue des Nations (F)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Moins que 126.5</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>09/07 03:00</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2.35</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>43,1%</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>+1,20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>45846.39348122294</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Paris SG – Real MadridInternational - Coupe du Monde des Clubs 2025</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Moins que 24.5 - tirs</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>09/07 19:00</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>36,1%</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>+1,04%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 10:24:54
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2148,7 +2148,7 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>45846.39348122294</v>
+        <v>45846.39348122685</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2170,10 +2170,8 @@
           <t>08/07 11:30</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>1.72</t>
-        </is>
+      <c r="F46" t="n">
+        <v>1.72</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2188,7 +2186,7 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>45846.39348122294</v>
+        <v>45846.39348122685</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2210,10 +2208,8 @@
           <t>09/07 03:00</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>2.35</t>
-        </is>
+      <c r="F47" t="n">
+        <v>2.35</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2228,7 +2224,7 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>45846.39348122294</v>
+        <v>45846.39348122685</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2250,10 +2246,8 @@
           <t>09/07 19:00</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>2.80</t>
-        </is>
+      <c r="F48" t="n">
+        <v>2.8</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2263,6 +2257,286 @@
       <c r="H48" t="inlineStr">
         <is>
           <t>+1,04%</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>45846.43385312291</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Metaloglobus Bucuresti – FC Universitatea ClujLiga 1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Plus que 3.51re équipe</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>11/07 16:00</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2,17%</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>+30,4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>45846.43385312291</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>FC Inter Turku – FF Jaro385076e7 Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Plus que 3.52e équipe</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>12/07 14:00</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2,07%</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>+24,2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>45846.43385312291</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Sportivo Ameliano – Cerro PortenoPrimera Division A9ZJ2X7R 385076e7</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Plus que 3.51re équipe</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>12/07 18:30</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2,90%</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>+16,2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>45846.43385312291</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Pologne F. – Suède F.Europe - Euro Féminin 2025</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Pénalité marquée: Non</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>74,4%</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>+5,69%</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>45846.43385312291</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Jannik Sinner – Ben SheltonWimbledon (H)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Plus que 6.51er set1er participant</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>09/07 10:00</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>24,6%</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>+3,42%</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>45846.43385312291</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PMU(FR)Football</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>KF Drita – Differdange 03Europe. Ligue des Champions (Q)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>11-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>08/07 18:00</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>1.44</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>71,8%</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>+3,34%</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>45846.43385312291</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PMU(FR)Football</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Levadia Tallinn – Rigas Futbola SkolaEurope. Ligue des Champions (Q)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>21-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>08/07 16:30</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>1.19</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>84,7%</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>+0,75%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 11:20:20
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2262,7 +2262,7 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>45846.43385312291</v>
+        <v>45846.433853125</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2284,10 +2284,8 @@
           <t>11/07 16:00</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
+      <c r="F49" t="n">
+        <v>60</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2302,7 +2300,7 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>45846.43385312291</v>
+        <v>45846.433853125</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2324,10 +2322,8 @@
           <t>12/07 14:00</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
+      <c r="F50" t="n">
+        <v>60</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2342,7 +2338,7 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>45846.43385312291</v>
+        <v>45846.433853125</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -2364,10 +2360,8 @@
           <t>12/07 18:30</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F51" t="n">
+        <v>40</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2382,7 +2376,7 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>45846.43385312291</v>
+        <v>45846.433853125</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -2404,10 +2398,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>1.42</t>
-        </is>
+      <c r="F52" t="n">
+        <v>1.42</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2422,7 +2414,7 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>45846.43385312291</v>
+        <v>45846.433853125</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -2444,10 +2436,8 @@
           <t>09/07 10:00</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
+      <c r="F53" t="n">
+        <v>4.2</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2462,7 +2452,7 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>45846.43385312291</v>
+        <v>45846.433853125</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -2484,10 +2474,8 @@
           <t>08/07 18:00</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>1.44</t>
-        </is>
+      <c r="F54" t="n">
+        <v>1.44</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2502,7 +2490,7 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>45846.43385312291</v>
+        <v>45846.433853125</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -2524,10 +2512,8 @@
           <t>08/07 16:30</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>1.19</t>
-        </is>
+      <c r="F55" t="n">
+        <v>1.19</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2537,6 +2523,206 @@
       <c r="H55" t="inlineStr">
         <is>
           <t>+0,75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>45846.47235413034</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Sportivo Ameliano – Cerro Porteno385076e7 Primera Division</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Plus que 3.51re équipe</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>12/07 18:30</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2,90%</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>+16,2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>45846.47235413034</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PokerStars(FR)Basketball</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Chicago Sky – Washington MysticsUSA - WNBA (ADJ98280) 385076e7</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>X2e période[race to 15 regular time]</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>08/07 15:30</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>25.00</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>4,28%</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>+6,89%</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>45846.47235413034</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Allemagne F. – Danemark F.Europe - Euro Féminin 2025</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Pénalité marquée: Non</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>08/07 16:00</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>73,4%</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>+6,42%</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>45846.47235413034</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>KF Egnatia Rrogozhine – BreidablikLigue des Champions</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Plus que 3.52e équipe</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>45.00</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2,32%</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>+4,30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>45846.47235413034</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>PMU(FR)Football</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>FC Noah Yerevan – Buducnost PodgoricaEurope. Ligue des Champions (Q)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>11-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>08/07 16:00</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>82,6%</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>+2,43%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 12:47:18
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2528,7 +2528,7 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>45846.47235413034</v>
+        <v>45846.47235413195</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -2550,10 +2550,8 @@
           <t>12/07 18:30</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F56" t="n">
+        <v>40</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2568,7 +2566,7 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>45846.47235413034</v>
+        <v>45846.47235413195</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -2590,10 +2588,8 @@
           <t>08/07 15:30</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>25.00</t>
-        </is>
+      <c r="F57" t="n">
+        <v>25</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2608,7 +2604,7 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>45846.47235413034</v>
+        <v>45846.47235413195</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -2630,10 +2626,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>1.45</t>
-        </is>
+      <c r="F58" t="n">
+        <v>1.45</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2648,7 +2642,7 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>45846.47235413034</v>
+        <v>45846.47235413195</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -2670,10 +2664,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F59" t="n">
+        <v>45</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2688,7 +2680,7 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>45846.47235413034</v>
+        <v>45846.47235413195</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -2710,10 +2702,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>1.24</t>
-        </is>
+      <c r="F60" t="n">
+        <v>1.24</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2723,6 +2713,166 @@
       <c r="H60" t="inlineStr">
         <is>
           <t>+2,43%</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>45846.53273709529</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Pologne – SuèdeUEFA Euro (F) - Matchs</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Plus que 3.51re équipe</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>140.00</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2,95%</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>+313%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>45846.53273709529</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>PokerStars(FR)Basketball</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Chicago Sky – Washington MysticsUSA - WNBA A9ZJ2X7R 385076e7</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>X2e période[race to 15 regular time]</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>08/07 15:30</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>25.00</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>4,23%</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>+5,78%</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>45846.53273709529</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Volleyball</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Bulgarie (F) – Brésil (F)International - Ligue des Nations (F)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>H 2 (−21.5)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>09/07 03:00</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>61,3%</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>+1,73%</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>45846.53273709529</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Amanda Anisimova – Anastasia PavlyuchenkovaWimbledon (F)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>1 - aces</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>08/07 13:40</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>1.70</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>59,2%</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>+0,65%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 13:36:25
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2718,7 +2718,7 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>45846.53273709529</v>
+        <v>45846.53273709491</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -2740,10 +2740,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>140.00</t>
-        </is>
+      <c r="F61" t="n">
+        <v>140</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2758,7 +2756,7 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>45846.53273709529</v>
+        <v>45846.53273709491</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -2780,10 +2778,8 @@
           <t>08/07 15:30</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>25.00</t>
-        </is>
+      <c r="F62" t="n">
+        <v>25</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2798,7 +2794,7 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>45846.53273709529</v>
+        <v>45846.53273709491</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -2820,10 +2816,8 @@
           <t>09/07 03:00</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>1.66</t>
-        </is>
+      <c r="F63" t="n">
+        <v>1.66</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2838,7 +2832,7 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>45846.53273709529</v>
+        <v>45846.53273709491</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -2860,10 +2854,8 @@
           <t>08/07 13:40</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>1.70</t>
-        </is>
+      <c r="F64" t="n">
+        <v>1.7</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2873,6 +2865,46 @@
       <c r="H64" t="inlineStr">
         <is>
           <t>+0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>45846.56686018862</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>PokerStars(FR)Basketball</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Chicago Sky – Washington MysticsUSA - WNBA</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>X2e période[race to 15 regular time]</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>08/07 15:30</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>25.00</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>4,41%</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>+10,4%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 14:21:53
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2870,7 +2870,7 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>45846.56686018862</v>
+        <v>45846.56686018519</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -2892,10 +2892,8 @@
           <t>08/07 15:30</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>25.00</t>
-        </is>
+      <c r="F65" t="n">
+        <v>25</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2905,6 +2903,126 @@
       <c r="H65" t="inlineStr">
         <is>
           <t>+10,4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>45846.59847204623</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Shelbourne FC – LinfieldEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>11-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>09/07 18:45</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2.20</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>46,3%</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>+1,86%</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>45846.59847204623</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Jannik Sinner – Ben SheltonWimbledon (H)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Moins que 4.51er set1er participant</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>09/07 13:10</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>5.20</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>19,3%</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>+0,19%</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>45846.59847204623</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Paris SG – Real MadridCoupe du Monde des Clubs</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Remplaçant marque un but: Oui</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>09/07 19:00</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>40,0%</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>+0,05%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 15:25:05
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2908,7 +2908,7 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>45846.59847204623</v>
+        <v>45846.59847204861</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -2930,10 +2930,8 @@
           <t>09/07 18:45</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>2.20</t>
-        </is>
+      <c r="F66" t="n">
+        <v>2.2</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2948,7 +2946,7 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>45846.59847204623</v>
+        <v>45846.59847204861</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -2970,10 +2968,8 @@
           <t>09/07 13:10</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>5.20</t>
-        </is>
+      <c r="F67" t="n">
+        <v>5.2</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2988,7 +2984,7 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>45846.59847204623</v>
+        <v>45846.59847204861</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -3010,10 +3006,8 @@
           <t>09/07 19:00</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>2.50</t>
-        </is>
+      <c r="F68" t="n">
+        <v>2.5</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -3023,6 +3017,46 @@
       <c r="H68" t="inlineStr">
         <is>
           <t>+0,05%</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>45846.64233208888</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Bwin(FR)Football</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Fotbal Club FCSB – Inter Club d'EscaldesEurope - Ligue des Champions stq pr cu 385076e7</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>2 / HNB</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>09/07 17:30</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>4.33</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>23,8%</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>+3,18%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 16:30:01
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3022,7 +3022,7 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>45846.64233208888</v>
+        <v>45846.64233208333</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -3044,10 +3044,8 @@
           <t>09/07 17:30</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
+      <c r="F69" t="n">
+        <v>4.33</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -3057,6 +3055,126 @@
       <c r="H69" t="inlineStr">
         <is>
           <t>+3,18%</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>45846.68740866632</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Paris SG – Real MadridInternational - Coupe du Monde des Clubs 2025 (ADJ98280) 385076e7</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Moins que 24.5 - tirs</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>09/07 19:00</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>36,1%</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>+15,6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>45846.68740866632</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Olimpija Ljubljana – Kairat AlmatyEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>21-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>08/07 17:00</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2.40</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>43,1%</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>+3,33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>45846.68740866632</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>PokerStars(FR)Basketball</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries – Indiana FeverUSA - WNBA</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>X2e période[race to 15 regular time]</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>09/07 16:00</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>25.00</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>4,02%</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>+0,48%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 17:20:50
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3060,7 +3060,7 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>45846.68740866632</v>
+        <v>45846.68740866898</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -3082,10 +3082,8 @@
           <t>09/07 19:00</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
+      <c r="F70" t="n">
+        <v>3.2</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -3100,7 +3098,7 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>45846.68740866632</v>
+        <v>45846.68740866898</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -3122,10 +3120,8 @@
           <t>08/07 17:00</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>2.40</t>
-        </is>
+      <c r="F71" t="n">
+        <v>2.4</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -3140,7 +3136,7 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>45846.68740866632</v>
+        <v>45846.68740866898</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -3162,10 +3158,8 @@
           <t>09/07 16:00</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>25.00</t>
-        </is>
+      <c r="F72" t="n">
+        <v>25</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -3175,6 +3169,86 @@
       <c r="H72" t="inlineStr">
         <is>
           <t>+0,48%</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>45846.72271245205</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>KF Egnatia Rrogozhine – BreidablikLigue des Champions - YYUZJR 385076e7</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Plus que 3.52e équipe</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>50.00</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2,21%</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>+10,5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>45846.72271245205</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>PMU(FR)Football</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Shelbourne FC – Linfield FCEurope. Ligue des Champions (Q)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>11-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>09/07 18:45</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>48,9%</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>+2,59%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 18:32:13
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3174,7 +3174,7 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>45846.72271245205</v>
+        <v>45846.7227124537</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -3196,10 +3196,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>50.00</t>
-        </is>
+      <c r="F73" t="n">
+        <v>50</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -3214,7 +3212,7 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>45846.72271245205</v>
+        <v>45846.7227124537</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -3236,19 +3234,97 @@
           <t>09/07 18:45</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F74" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>48,9%</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>+2,59%</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>45846.77230864445</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Football</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Fluminense – ChelseaInternational - CDM des Clubs</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Moins que 24.5 - tirs</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
         <is>
           <t>2.10</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>48,9%</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>+2,59%</t>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>49,3%</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>+3,56%</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>45846.77230864445</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>PMU(FR)Football</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Ludogorets Razgrad – Dinamo MinskEurope. Ligue des Champions (Q)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>11-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>09/07 17:30</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>80,6%</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>+1,55%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 19:18:21
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3250,7 +3250,7 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>45846.77230864445</v>
+        <v>45846.77230864584</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -3272,10 +3272,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
+      <c r="F75" t="n">
+        <v>2.1</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3290,7 +3288,7 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>45846.77230864445</v>
+        <v>45846.77230864584</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -3312,10 +3310,8 @@
           <t>09/07 17:30</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>1.26</t>
-        </is>
+      <c r="F76" t="n">
+        <v>1.26</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3325,6 +3321,86 @@
       <c r="H76" t="inlineStr">
         <is>
           <t>+1,55%</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>45846.8043397411</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Volleyball</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Bulgarie (F) – Brésil (F)International - Ligue des Nations (F)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Moins que 132.5</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>09/07 03:00</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>66,0%</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>+2,88%</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>45846.8043397411</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>IA Akranes – KR ReykjavikIslande - Islande Úrvalsdeild</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Pas de buts</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>14/07 19:15</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2,53%</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>+1,32%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 20:25:38
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3326,7 +3326,7 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>45846.8043397411</v>
+        <v>45846.80433974537</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -3348,10 +3348,8 @@
           <t>09/07 03:00</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>1.56</t>
-        </is>
+      <c r="F77" t="n">
+        <v>1.56</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3366,7 +3364,7 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>45846.8043397411</v>
+        <v>45846.80433974537</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -3388,10 +3386,8 @@
           <t>14/07 19:15</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F78" t="n">
+        <v>40</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -3401,6 +3397,126 @@
       <c r="H78" t="inlineStr">
         <is>
           <t>+1,32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>45846.85106990638</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>PMU(FR)Volleyball</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Bulgarie (F) – Brésil (F)Volleyball. Ligue des Nations (F)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Plus que 40.51er set</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>09/07 03:00</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>66,1%</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>+7,75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>45846.85106990638</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>PMU(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Fritz, Taylor – Alcaraz, CarlosEvénements. Wimbledon (H)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Moins que 8.51er set</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>09/07 09:00</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>6.50</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>16,2%</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>+5,12%</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>45846.85106990638</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>PMU(FR)Football</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Vilnius Zalgiris – Hamrun SpartansEurope. Ligue des Champions (Q)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>11-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>09/07 16:00</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>56,1%</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>+2,65%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 22:47:50
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -498,10 +498,8 @@
           <t>11/07 18:00</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
+      <c r="F2" t="n">
+        <v>60</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -516,7 +514,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -538,10 +536,8 @@
           <t>11/07 23:30</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>55.00</t>
-        </is>
+      <c r="F3" t="n">
+        <v>55</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -556,7 +552,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -578,10 +574,8 @@
           <t>12/07 16:00</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
+      <c r="F4" t="n">
+        <v>60</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -596,7 +590,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -618,10 +612,8 @@
           <t>12/07 23:00</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F5" t="n">
+        <v>45</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -636,7 +628,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -658,10 +650,8 @@
           <t>09/07 21:00</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>3.15</t>
-        </is>
+      <c r="F6" t="n">
+        <v>3.15</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -676,7 +666,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -698,10 +688,8 @@
           <t>09/07 15:10</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>5.20</t>
-        </is>
+      <c r="F7" t="n">
+        <v>5.2</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -716,7 +704,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -738,10 +726,8 @@
           <t>12/07 21:00</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F8" t="n">
+        <v>45</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -756,7 +742,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -778,10 +764,8 @@
           <t>12/07 17:30</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>50.00</t>
-        </is>
+      <c r="F9" t="n">
+        <v>50</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -796,7 +780,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -818,10 +802,8 @@
           <t>09/07 05:00</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>1.63</t>
-        </is>
+      <c r="F10" t="n">
+        <v>1.63</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -836,7 +818,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -858,10 +840,8 @@
           <t>09/07 20:45</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
+      <c r="F11" t="n">
+        <v>2.1</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -876,7 +856,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -898,10 +878,8 @@
           <t>12/07 20:30</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F12" t="n">
+        <v>40</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -916,7 +894,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -938,10 +916,8 @@
           <t>09/07 18:00</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
+      <c r="F13" t="n">
+        <v>1.83</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -956,7 +932,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -978,10 +954,8 @@
           <t>09/07 19:30</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>1.26</t>
-        </is>
+      <c r="F14" t="n">
+        <v>1.26</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -996,7 +970,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1018,10 +992,8 @@
           <t>09/07 19:30</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>1.04</t>
-        </is>
+      <c r="F15" t="n">
+        <v>1.04</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1036,7 +1008,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45846.94871857774</v>
+        <v>45846.94871857639</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1058,10 +1030,8 @@
           <t>14/07 21:15</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F16" t="n">
+        <v>40</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1071,6 +1041,46 @@
       <c r="H16" t="inlineStr">
         <is>
           <t>+0,04%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>45846.94975841979</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>New England Revolution – Inter Miami CFÉtats-Unis - États-Unis MLS</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Moins que 8.5 - tir cadré</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>10/07 01:30</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2.65</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>40,3%</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>+6,72%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour des données valuebets
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,6 +473,11 @@
           <t>overvalue</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>event_short</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -511,6 +516,11 @@
           <t>+42,9%</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Metaloglob</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -549,6 +559,11 @@
           <t>+28,7%</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>CS 2 de Ma</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -587,6 +602,11 @@
           <t>+25,0%</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>FC Inter T</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -625,6 +645,11 @@
           <t>+18,3%</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Nacional A</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -663,6 +688,11 @@
           <t>+18,2%</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Paris SG –</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -701,6 +731,11 @@
           <t>+17,2%</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Jannik Sin</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -739,6 +774,11 @@
           <t>+12,1%</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>AD Pasto –</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -777,6 +817,11 @@
           <t>+9,33%</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Malmo FF –</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -815,6 +860,11 @@
           <t>+6,36%</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Bulgarie (</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -853,6 +903,11 @@
           <t>+4,46%</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Shelbourne</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -891,6 +946,11 @@
           <t>+3,52%</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Sportivo A</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -929,6 +989,11 @@
           <t>+3,29%</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Vilnius Za</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -967,6 +1032,11 @@
           <t>+2,78%</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Ludogorets</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1005,6 +1075,11 @@
           <t>+0,81%</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>FCSB – Int</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1043,10 +1118,15 @@
           <t>+0,04%</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>IA Akranes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>45846.94975841979</v>
+        <v>45846.94975841435</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1068,10 +1148,8 @@
           <t>10/07 01:30</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>2.65</t>
-        </is>
+      <c r="F17" t="n">
+        <v>2.65</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1081,6 +1159,146 @@
       <c r="H17" t="inlineStr">
         <is>
           <t>+6,72%</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>New Englan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>45846.97293791649</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Jannik Sinner – Ben SheltonWimbledon (H)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Moins que 5.51er set1er participant</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>09/07 15:10</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>24,5%</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>+10,1%</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Jannik Sin</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>45846.97293791649</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PMU(FR)Football</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Vilnius Zalgiris – Hamrun SpartansEurope. Ligue des Champions (Q)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>09/07 18:00</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>5.80</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>18,0%</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>+4,43%</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Vilnius Za</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>45846.97293791649</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Volleyball</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Bulgarie (F) – Brésil (F)International - Ligue des Nations (F)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Moins que 132.5</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>09/07 05:00</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>66,0%</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>+2,89%</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Bulgarie (</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-08 21:21:39
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-08.xlsx
+++ b/data/valuebets_database_2025-07-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3402,7 +3402,7 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>45846.85106990638</v>
+        <v>45846.85106990741</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -3424,10 +3424,8 @@
           <t>09/07 03:00</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>1.63</t>
-        </is>
+      <c r="F79" t="n">
+        <v>1.63</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -3442,7 +3440,7 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>45846.85106990638</v>
+        <v>45846.85106990741</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -3464,10 +3462,8 @@
           <t>09/07 09:00</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>6.50</t>
-        </is>
+      <c r="F80" t="n">
+        <v>6.5</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -3482,7 +3478,7 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>45846.85106990638</v>
+        <v>45846.85106990741</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -3504,10 +3500,8 @@
           <t>09/07 16:00</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
+      <c r="F81" t="n">
+        <v>1.83</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -3517,6 +3511,86 @@
       <c r="H81" t="inlineStr">
         <is>
           <t>+2,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>45846.88992982436</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Tennis</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Jannik Sinner – Ben SheltonWimbledon (H)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Moins que 5.51er set1er participant</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>09/07 13:10</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>24,5%</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>+10,1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>45846.88992982436</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>PMU(FR)Football</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Vilnius Zalgiris – Hamrun SpartansEurope. Ligue des Champions (Q)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>09/07 16:00</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>5.80</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>18,0%</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>+4,48%</t>
         </is>
       </c>
     </row>

</xml_diff>